<commit_message>
Agrego graficos nativos de dispersion y tablas de coordenadas manteniendo imagenes graficas en Excel
</commit_message>
<xml_diff>
--- a/Casos_Particulares_Guia_PLC_Consignas.xlsx
+++ b/Casos_Particulares_Guia_PLC_Consignas.xlsx
@@ -19,7 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="7">
     <font>
       <name val="Calibri"/>
@@ -172,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -214,6 +216,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -313,6 +318,798 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Gráfico Nativo Interactivo de Excel (Ejercicio 4.7)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'4.7 - Alternativas'!M26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.7 - Alternativas'!$L$27:$L$32</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.7 - Alternativas'!$M$27:$M$32</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'4.7 - Alternativas'!N26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.7 - Alternativas'!$L$27:$L$32</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.7 - Alternativas'!$N$27:$N$32</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'4.7 - Alternativas'!O26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.7 - Alternativas'!$L$27:$L$32</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.7 - Alternativas'!$O$27:$O$32</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'4.7 - Alternativas'!P26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.7 - Alternativas'!$L$27:$L$32</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.7 - Alternativas'!$P$27:$P$32</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>x1 (Mesas de Pino)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>x2 (Mesas de Roble)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Gráfico Nativo Interactivo de Excel (Ejercicio 4.8)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'4.8 - Degenerada'!M26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.8 - Degenerada'!$L$27:$L$31</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.8 - Degenerada'!$M$27:$M$31</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'4.8 - Degenerada'!N26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.8 - Degenerada'!$L$27:$L$31</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.8 - Degenerada'!$N$27:$N$31</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'4.8 - Degenerada'!O26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.8 - Degenerada'!$L$27:$L$31</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.8 - Degenerada'!$O$27:$O$31</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'4.8 - Degenerada'!P26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.8 - Degenerada'!$L$27:$L$31</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.8 - Degenerada'!$P$27:$P$31</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>x1 (Fertilizante N-Plus)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>x2 (Fertilizante P-Max)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Gráfico Nativo Interactivo de Excel (Ejercicio 4.10 - No Acotada)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'4.10 - No Acotada'!M26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.10 - No Acotada'!$L$27:$L$31</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.10 - No Acotada'!$M$27:$M$31</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'4.10 - No Acotada'!N26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.10 - No Acotada'!$L$27:$L$31</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.10 - No Acotada'!$N$27:$N$31</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'4.10 - No Acotada'!O26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.10 - No Acotada'!$L$27:$L$31</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.10 - No Acotada'!$O$27:$O$31</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>x1 (PET Reciclado)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>x2 (Polietileno)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Gráfico Nativo Interactivo de Excel (Ejercicio 4.12 - Incompatible)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'4.12 - Incompatible'!M26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.12 - Incompatible'!$L$27:$L$30</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.12 - Incompatible'!$M$27:$M$30</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'4.12 - Incompatible'!N26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.12 - Incompatible'!$L$27:$L$30</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.12 - Incompatible'!$N$27:$N$30</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'4.12 - Incompatible'!O26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'4.12 - Incompatible'!$L$27:$L$30</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'4.12 - Incompatible'!$O$27:$O$30</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>x1 (Camisas)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>x2 (Pantalones)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -399,7 +1196,29 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
   <oneCellAnchor>
     <from>
       <col>11</col>
@@ -407,14 +1226,14 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="3524250"/>
+    <ext cx="4095750" cy="3286125"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -429,7 +1248,29 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
   <oneCellAnchor>
     <from>
       <col>11</col>
@@ -437,14 +1278,14 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="3524250"/>
+    <ext cx="4095750" cy="3286125"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -459,7 +1300,29 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
   <oneCellAnchor>
     <from>
       <col>11</col>
@@ -467,14 +1330,14 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="3524250"/>
+    <ext cx="4095750" cy="3286125"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -489,7 +1352,29 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3960000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
   <oneCellAnchor>
     <from>
       <col>11</col>
@@ -497,14 +1382,14 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="3524250"/>
+    <ext cx="4095750" cy="3286125"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip cstate="print" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -807,7 +1692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -820,6 +1705,12 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -1114,14 +2005,58 @@
         <v/>
       </c>
       <c r="J25" s="16" t="n"/>
-    </row>
-    <row r="26"/>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>TABLA DE PUNTOS PARA EL GRÁFICO NATIVO DE EXCEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="L26" s="19" t="inlineStr">
+        <is>
+          <t>x_val</t>
+        </is>
+      </c>
+      <c r="M26" s="19" t="inlineStr">
+        <is>
+          <t>R1 (x1&lt;=6)</t>
+        </is>
+      </c>
+      <c r="N26" s="19" t="inlineStr">
+        <is>
+          <t>R2 (x1+x2&lt;=8)</t>
+        </is>
+      </c>
+      <c r="O26" s="19" t="inlineStr">
+        <is>
+          <t>R3 (x1+2x2&lt;=12)</t>
+        </is>
+      </c>
+      <c r="P26" s="19" t="inlineStr">
+        <is>
+          <t>Segmento Opt (Z=32)</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
           <t>PRIMERA TABLA ÓPTIMA (TOP 1) - Vértice A: (6 mesas de pino, 2 mesas de roble)</t>
         </is>
       </c>
+      <c r="L27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="N27" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="O27" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="P27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr"/>
@@ -1153,6 +2088,21 @@
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr"/>
+      <c r="L28" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="M28" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="N28" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="O28" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="P28" s="20" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="19" t="inlineStr">
@@ -1199,6 +2149,21 @@
         <is>
           <t>Θ</t>
         </is>
+      </c>
+      <c r="L29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="M29" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="N29" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="O29" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="P29" s="20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -1233,6 +2198,19 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L30" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="M30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="O30" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="P30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="8" t="n">
@@ -1265,6 +2243,17 @@
         <f>D31/I31</f>
         <v/>
       </c>
+      <c r="L31" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="M31" s="10" t="n"/>
+      <c r="N31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="P31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="8" t="n">
@@ -1298,6 +2287,15 @@
           <t>-</t>
         </is>
       </c>
+      <c r="L32" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="M32" s="10" t="n"/>
+      <c r="N32" s="10" t="n"/>
+      <c r="O32" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="12" t="inlineStr">
@@ -1310,7 +2308,7 @@
           <t>=</t>
         </is>
       </c>
-      <c r="D33" s="20">
+      <c r="D33" s="21">
         <f>B30*D30+B31*D31+B32*D32</f>
         <v/>
       </c>
@@ -1349,7 +2347,7 @@
         <f>B$30*H30+B$31*H31+B$32*H32-H$28</f>
         <v/>
       </c>
-      <c r="I34" s="21">
+      <c r="I34" s="22">
         <f>B$30*I30+B$31*I31+B$32*I32-I$28</f>
         <v/>
       </c>
@@ -1551,7 +2549,7 @@
           <t>=</t>
         </is>
       </c>
-      <c r="D42" s="20">
+      <c r="D42" s="21">
         <f>B39*D39+B40*D40+B41*D41</f>
         <v/>
       </c>
@@ -1606,7 +2604,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B47" s="23" t="inlineStr">
         <is>
           <t>• Respuesta a) Formulación Deducida:
    Variables: X1 = Mesas de pino por semana | X2 = Mesas de roble por semana.
@@ -1622,157 +2620,157 @@
    5. Causa Geométrica: La pendiente del funcional (m = -4/4 = -1) es paralela a la restricción activa de armado (m = -1/1 = -1).</t>
         </is>
       </c>
-      <c r="C47" s="23" t="n"/>
-      <c r="D47" s="23" t="n"/>
-      <c r="E47" s="23" t="n"/>
-      <c r="F47" s="23" t="n"/>
-      <c r="G47" s="23" t="n"/>
-      <c r="H47" s="23" t="n"/>
-      <c r="I47" s="23" t="n"/>
-      <c r="J47" s="23" t="n"/>
+      <c r="C47" s="24" t="n"/>
+      <c r="D47" s="24" t="n"/>
+      <c r="E47" s="24" t="n"/>
+      <c r="F47" s="24" t="n"/>
+      <c r="G47" s="24" t="n"/>
+      <c r="H47" s="24" t="n"/>
+      <c r="I47" s="24" t="n"/>
+      <c r="J47" s="24" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="23" t="n"/>
-      <c r="C48" s="23" t="n"/>
-      <c r="D48" s="23" t="n"/>
-      <c r="E48" s="23" t="n"/>
-      <c r="F48" s="23" t="n"/>
-      <c r="G48" s="23" t="n"/>
-      <c r="H48" s="23" t="n"/>
-      <c r="I48" s="23" t="n"/>
-      <c r="J48" s="23" t="n"/>
+      <c r="B48" s="24" t="n"/>
+      <c r="C48" s="24" t="n"/>
+      <c r="D48" s="24" t="n"/>
+      <c r="E48" s="24" t="n"/>
+      <c r="F48" s="24" t="n"/>
+      <c r="G48" s="24" t="n"/>
+      <c r="H48" s="24" t="n"/>
+      <c r="I48" s="24" t="n"/>
+      <c r="J48" s="24" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="23" t="n"/>
-      <c r="C49" s="23" t="n"/>
-      <c r="D49" s="23" t="n"/>
-      <c r="E49" s="23" t="n"/>
-      <c r="F49" s="23" t="n"/>
-      <c r="G49" s="23" t="n"/>
-      <c r="H49" s="23" t="n"/>
-      <c r="I49" s="23" t="n"/>
-      <c r="J49" s="23" t="n"/>
+      <c r="B49" s="24" t="n"/>
+      <c r="C49" s="24" t="n"/>
+      <c r="D49" s="24" t="n"/>
+      <c r="E49" s="24" t="n"/>
+      <c r="F49" s="24" t="n"/>
+      <c r="G49" s="24" t="n"/>
+      <c r="H49" s="24" t="n"/>
+      <c r="I49" s="24" t="n"/>
+      <c r="J49" s="24" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="23" t="n"/>
-      <c r="C50" s="23" t="n"/>
-      <c r="D50" s="23" t="n"/>
-      <c r="E50" s="23" t="n"/>
-      <c r="F50" s="23" t="n"/>
-      <c r="G50" s="23" t="n"/>
-      <c r="H50" s="23" t="n"/>
-      <c r="I50" s="23" t="n"/>
-      <c r="J50" s="23" t="n"/>
+      <c r="B50" s="24" t="n"/>
+      <c r="C50" s="24" t="n"/>
+      <c r="D50" s="24" t="n"/>
+      <c r="E50" s="24" t="n"/>
+      <c r="F50" s="24" t="n"/>
+      <c r="G50" s="24" t="n"/>
+      <c r="H50" s="24" t="n"/>
+      <c r="I50" s="24" t="n"/>
+      <c r="J50" s="24" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="23" t="n"/>
-      <c r="C51" s="23" t="n"/>
-      <c r="D51" s="23" t="n"/>
-      <c r="E51" s="23" t="n"/>
-      <c r="F51" s="23" t="n"/>
-      <c r="G51" s="23" t="n"/>
-      <c r="H51" s="23" t="n"/>
-      <c r="I51" s="23" t="n"/>
-      <c r="J51" s="23" t="n"/>
+      <c r="B51" s="24" t="n"/>
+      <c r="C51" s="24" t="n"/>
+      <c r="D51" s="24" t="n"/>
+      <c r="E51" s="24" t="n"/>
+      <c r="F51" s="24" t="n"/>
+      <c r="G51" s="24" t="n"/>
+      <c r="H51" s="24" t="n"/>
+      <c r="I51" s="24" t="n"/>
+      <c r="J51" s="24" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="23" t="n"/>
-      <c r="C52" s="23" t="n"/>
-      <c r="D52" s="23" t="n"/>
-      <c r="E52" s="23" t="n"/>
-      <c r="F52" s="23" t="n"/>
-      <c r="G52" s="23" t="n"/>
-      <c r="H52" s="23" t="n"/>
-      <c r="I52" s="23" t="n"/>
-      <c r="J52" s="23" t="n"/>
+      <c r="B52" s="24" t="n"/>
+      <c r="C52" s="24" t="n"/>
+      <c r="D52" s="24" t="n"/>
+      <c r="E52" s="24" t="n"/>
+      <c r="F52" s="24" t="n"/>
+      <c r="G52" s="24" t="n"/>
+      <c r="H52" s="24" t="n"/>
+      <c r="I52" s="24" t="n"/>
+      <c r="J52" s="24" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="23" t="n"/>
-      <c r="C53" s="23" t="n"/>
-      <c r="D53" s="23" t="n"/>
-      <c r="E53" s="23" t="n"/>
-      <c r="F53" s="23" t="n"/>
-      <c r="G53" s="23" t="n"/>
-      <c r="H53" s="23" t="n"/>
-      <c r="I53" s="23" t="n"/>
-      <c r="J53" s="23" t="n"/>
+      <c r="B53" s="24" t="n"/>
+      <c r="C53" s="24" t="n"/>
+      <c r="D53" s="24" t="n"/>
+      <c r="E53" s="24" t="n"/>
+      <c r="F53" s="24" t="n"/>
+      <c r="G53" s="24" t="n"/>
+      <c r="H53" s="24" t="n"/>
+      <c r="I53" s="24" t="n"/>
+      <c r="J53" s="24" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="23" t="n"/>
-      <c r="C54" s="23" t="n"/>
-      <c r="D54" s="23" t="n"/>
-      <c r="E54" s="23" t="n"/>
-      <c r="F54" s="23" t="n"/>
-      <c r="G54" s="23" t="n"/>
-      <c r="H54" s="23" t="n"/>
-      <c r="I54" s="23" t="n"/>
-      <c r="J54" s="23" t="n"/>
+      <c r="B54" s="24" t="n"/>
+      <c r="C54" s="24" t="n"/>
+      <c r="D54" s="24" t="n"/>
+      <c r="E54" s="24" t="n"/>
+      <c r="F54" s="24" t="n"/>
+      <c r="G54" s="24" t="n"/>
+      <c r="H54" s="24" t="n"/>
+      <c r="I54" s="24" t="n"/>
+      <c r="J54" s="24" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="23" t="n"/>
-      <c r="C55" s="23" t="n"/>
-      <c r="D55" s="23" t="n"/>
-      <c r="E55" s="23" t="n"/>
-      <c r="F55" s="23" t="n"/>
-      <c r="G55" s="23" t="n"/>
-      <c r="H55" s="23" t="n"/>
-      <c r="I55" s="23" t="n"/>
-      <c r="J55" s="23" t="n"/>
+      <c r="B55" s="24" t="n"/>
+      <c r="C55" s="24" t="n"/>
+      <c r="D55" s="24" t="n"/>
+      <c r="E55" s="24" t="n"/>
+      <c r="F55" s="24" t="n"/>
+      <c r="G55" s="24" t="n"/>
+      <c r="H55" s="24" t="n"/>
+      <c r="I55" s="24" t="n"/>
+      <c r="J55" s="24" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="23" t="n"/>
-      <c r="C56" s="23" t="n"/>
-      <c r="D56" s="23" t="n"/>
-      <c r="E56" s="23" t="n"/>
-      <c r="F56" s="23" t="n"/>
-      <c r="G56" s="23" t="n"/>
-      <c r="H56" s="23" t="n"/>
-      <c r="I56" s="23" t="n"/>
-      <c r="J56" s="23" t="n"/>
+      <c r="B56" s="24" t="n"/>
+      <c r="C56" s="24" t="n"/>
+      <c r="D56" s="24" t="n"/>
+      <c r="E56" s="24" t="n"/>
+      <c r="F56" s="24" t="n"/>
+      <c r="G56" s="24" t="n"/>
+      <c r="H56" s="24" t="n"/>
+      <c r="I56" s="24" t="n"/>
+      <c r="J56" s="24" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="23" t="n"/>
-      <c r="C57" s="23" t="n"/>
-      <c r="D57" s="23" t="n"/>
-      <c r="E57" s="23" t="n"/>
-      <c r="F57" s="23" t="n"/>
-      <c r="G57" s="23" t="n"/>
-      <c r="H57" s="23" t="n"/>
-      <c r="I57" s="23" t="n"/>
-      <c r="J57" s="23" t="n"/>
+      <c r="B57" s="24" t="n"/>
+      <c r="C57" s="24" t="n"/>
+      <c r="D57" s="24" t="n"/>
+      <c r="E57" s="24" t="n"/>
+      <c r="F57" s="24" t="n"/>
+      <c r="G57" s="24" t="n"/>
+      <c r="H57" s="24" t="n"/>
+      <c r="I57" s="24" t="n"/>
+      <c r="J57" s="24" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="23" t="n"/>
-      <c r="C58" s="23" t="n"/>
-      <c r="D58" s="23" t="n"/>
-      <c r="E58" s="23" t="n"/>
-      <c r="F58" s="23" t="n"/>
-      <c r="G58" s="23" t="n"/>
-      <c r="H58" s="23" t="n"/>
-      <c r="I58" s="23" t="n"/>
-      <c r="J58" s="23" t="n"/>
+      <c r="B58" s="24" t="n"/>
+      <c r="C58" s="24" t="n"/>
+      <c r="D58" s="24" t="n"/>
+      <c r="E58" s="24" t="n"/>
+      <c r="F58" s="24" t="n"/>
+      <c r="G58" s="24" t="n"/>
+      <c r="H58" s="24" t="n"/>
+      <c r="I58" s="24" t="n"/>
+      <c r="J58" s="24" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="23" t="n"/>
-      <c r="C59" s="23" t="n"/>
-      <c r="D59" s="23" t="n"/>
-      <c r="E59" s="23" t="n"/>
-      <c r="F59" s="23" t="n"/>
-      <c r="G59" s="23" t="n"/>
-      <c r="H59" s="23" t="n"/>
-      <c r="I59" s="23" t="n"/>
-      <c r="J59" s="23" t="n"/>
+      <c r="B59" s="24" t="n"/>
+      <c r="C59" s="24" t="n"/>
+      <c r="D59" s="24" t="n"/>
+      <c r="E59" s="24" t="n"/>
+      <c r="F59" s="24" t="n"/>
+      <c r="G59" s="24" t="n"/>
+      <c r="H59" s="24" t="n"/>
+      <c r="I59" s="24" t="n"/>
+      <c r="J59" s="24" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="23" t="n"/>
-      <c r="C60" s="23" t="n"/>
-      <c r="D60" s="23" t="n"/>
-      <c r="E60" s="23" t="n"/>
-      <c r="F60" s="23" t="n"/>
-      <c r="G60" s="23" t="n"/>
-      <c r="H60" s="23" t="n"/>
-      <c r="I60" s="23" t="n"/>
-      <c r="J60" s="23" t="n"/>
+      <c r="B60" s="24" t="n"/>
+      <c r="C60" s="24" t="n"/>
+      <c r="D60" s="24" t="n"/>
+      <c r="E60" s="24" t="n"/>
+      <c r="F60" s="24" t="n"/>
+      <c r="G60" s="24" t="n"/>
+      <c r="H60" s="24" t="n"/>
+      <c r="I60" s="24" t="n"/>
+      <c r="J60" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1791,7 +2789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1804,6 +2802,12 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -2098,14 +3102,58 @@
         <v/>
       </c>
       <c r="J25" s="16" t="n"/>
-    </row>
-    <row r="26"/>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>TABLA DE PUNTOS PARA EL GRÁFICO NATIVO DE EXCEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="L26" s="19" t="inlineStr">
+        <is>
+          <t>x_val</t>
+        </is>
+      </c>
+      <c r="M26" s="19" t="inlineStr">
+        <is>
+          <t>R1 (2x1+4x2&lt;=48)</t>
+        </is>
+      </c>
+      <c r="N26" s="19" t="inlineStr">
+        <is>
+          <t>R2 (4x1+2x2&lt;=60)</t>
+        </is>
+      </c>
+      <c r="O26" s="19" t="inlineStr">
+        <is>
+          <t>R3 (3x1&lt;=45)</t>
+        </is>
+      </c>
+      <c r="P26" s="19" t="inlineStr">
+        <is>
+          <t>Vértice Óptimo (12, 6)</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
           <t>ITERACIÓN 1 - BASE DEGRADADA (Bk = 0 en λ3)</t>
         </is>
       </c>
+      <c r="L27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="N27" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="O27" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="P27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr"/>
@@ -2137,6 +3185,21 @@
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr"/>
+      <c r="L28" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="M28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="N28" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="O28" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="P28" s="20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="19" t="inlineStr">
@@ -2184,6 +3247,19 @@
           <t>Θ</t>
         </is>
       </c>
+      <c r="L29" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="M29" s="20" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="P29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="8" t="n">
@@ -2216,6 +3292,19 @@
         <f>D30/F30</f>
         <v/>
       </c>
+      <c r="L30" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="M30" s="20" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="8" t="n">
@@ -2248,6 +3337,15 @@
         <f>D31/F31</f>
         <v/>
       </c>
+      <c r="L31" s="20" t="n">
+        <v>24</v>
+      </c>
+      <c r="M31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="10" t="n"/>
+      <c r="O31" s="10" t="n"/>
+      <c r="P31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="8" t="n">
@@ -2258,7 +3356,7 @@
           <t>λ3</t>
         </is>
       </c>
-      <c r="D32" s="24" t="n">
+      <c r="D32" s="25" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="10" t="n">
@@ -2534,7 +3632,7 @@
           <t>=</t>
         </is>
       </c>
-      <c r="D42" s="20">
+      <c r="D42" s="21">
         <f>B39*D39+B40*D40+B41*D41</f>
         <v/>
       </c>
@@ -2589,7 +3687,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B47" s="23" t="inlineStr">
         <is>
           <t>• Respuesta a) Formulación Deducida:
    Variables: X1 = Litros mensuales de Fertilizante N-Plus | X2 = Litros mensuales de Fertilizante P-Max.
@@ -2607,157 +3705,157 @@
       y una holgura remanente de 9 minutos en la máquina de envasado (λ3 = 9).</t>
         </is>
       </c>
-      <c r="C47" s="23" t="n"/>
-      <c r="D47" s="23" t="n"/>
-      <c r="E47" s="23" t="n"/>
-      <c r="F47" s="23" t="n"/>
-      <c r="G47" s="23" t="n"/>
-      <c r="H47" s="23" t="n"/>
-      <c r="I47" s="23" t="n"/>
-      <c r="J47" s="23" t="n"/>
+      <c r="C47" s="24" t="n"/>
+      <c r="D47" s="24" t="n"/>
+      <c r="E47" s="24" t="n"/>
+      <c r="F47" s="24" t="n"/>
+      <c r="G47" s="24" t="n"/>
+      <c r="H47" s="24" t="n"/>
+      <c r="I47" s="24" t="n"/>
+      <c r="J47" s="24" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="23" t="n"/>
-      <c r="C48" s="23" t="n"/>
-      <c r="D48" s="23" t="n"/>
-      <c r="E48" s="23" t="n"/>
-      <c r="F48" s="23" t="n"/>
-      <c r="G48" s="23" t="n"/>
-      <c r="H48" s="23" t="n"/>
-      <c r="I48" s="23" t="n"/>
-      <c r="J48" s="23" t="n"/>
+      <c r="B48" s="24" t="n"/>
+      <c r="C48" s="24" t="n"/>
+      <c r="D48" s="24" t="n"/>
+      <c r="E48" s="24" t="n"/>
+      <c r="F48" s="24" t="n"/>
+      <c r="G48" s="24" t="n"/>
+      <c r="H48" s="24" t="n"/>
+      <c r="I48" s="24" t="n"/>
+      <c r="J48" s="24" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="23" t="n"/>
-      <c r="C49" s="23" t="n"/>
-      <c r="D49" s="23" t="n"/>
-      <c r="E49" s="23" t="n"/>
-      <c r="F49" s="23" t="n"/>
-      <c r="G49" s="23" t="n"/>
-      <c r="H49" s="23" t="n"/>
-      <c r="I49" s="23" t="n"/>
-      <c r="J49" s="23" t="n"/>
+      <c r="B49" s="24" t="n"/>
+      <c r="C49" s="24" t="n"/>
+      <c r="D49" s="24" t="n"/>
+      <c r="E49" s="24" t="n"/>
+      <c r="F49" s="24" t="n"/>
+      <c r="G49" s="24" t="n"/>
+      <c r="H49" s="24" t="n"/>
+      <c r="I49" s="24" t="n"/>
+      <c r="J49" s="24" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="23" t="n"/>
-      <c r="C50" s="23" t="n"/>
-      <c r="D50" s="23" t="n"/>
-      <c r="E50" s="23" t="n"/>
-      <c r="F50" s="23" t="n"/>
-      <c r="G50" s="23" t="n"/>
-      <c r="H50" s="23" t="n"/>
-      <c r="I50" s="23" t="n"/>
-      <c r="J50" s="23" t="n"/>
+      <c r="B50" s="24" t="n"/>
+      <c r="C50" s="24" t="n"/>
+      <c r="D50" s="24" t="n"/>
+      <c r="E50" s="24" t="n"/>
+      <c r="F50" s="24" t="n"/>
+      <c r="G50" s="24" t="n"/>
+      <c r="H50" s="24" t="n"/>
+      <c r="I50" s="24" t="n"/>
+      <c r="J50" s="24" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="23" t="n"/>
-      <c r="C51" s="23" t="n"/>
-      <c r="D51" s="23" t="n"/>
-      <c r="E51" s="23" t="n"/>
-      <c r="F51" s="23" t="n"/>
-      <c r="G51" s="23" t="n"/>
-      <c r="H51" s="23" t="n"/>
-      <c r="I51" s="23" t="n"/>
-      <c r="J51" s="23" t="n"/>
+      <c r="B51" s="24" t="n"/>
+      <c r="C51" s="24" t="n"/>
+      <c r="D51" s="24" t="n"/>
+      <c r="E51" s="24" t="n"/>
+      <c r="F51" s="24" t="n"/>
+      <c r="G51" s="24" t="n"/>
+      <c r="H51" s="24" t="n"/>
+      <c r="I51" s="24" t="n"/>
+      <c r="J51" s="24" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="23" t="n"/>
-      <c r="C52" s="23" t="n"/>
-      <c r="D52" s="23" t="n"/>
-      <c r="E52" s="23" t="n"/>
-      <c r="F52" s="23" t="n"/>
-      <c r="G52" s="23" t="n"/>
-      <c r="H52" s="23" t="n"/>
-      <c r="I52" s="23" t="n"/>
-      <c r="J52" s="23" t="n"/>
+      <c r="B52" s="24" t="n"/>
+      <c r="C52" s="24" t="n"/>
+      <c r="D52" s="24" t="n"/>
+      <c r="E52" s="24" t="n"/>
+      <c r="F52" s="24" t="n"/>
+      <c r="G52" s="24" t="n"/>
+      <c r="H52" s="24" t="n"/>
+      <c r="I52" s="24" t="n"/>
+      <c r="J52" s="24" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="23" t="n"/>
-      <c r="C53" s="23" t="n"/>
-      <c r="D53" s="23" t="n"/>
-      <c r="E53" s="23" t="n"/>
-      <c r="F53" s="23" t="n"/>
-      <c r="G53" s="23" t="n"/>
-      <c r="H53" s="23" t="n"/>
-      <c r="I53" s="23" t="n"/>
-      <c r="J53" s="23" t="n"/>
+      <c r="B53" s="24" t="n"/>
+      <c r="C53" s="24" t="n"/>
+      <c r="D53" s="24" t="n"/>
+      <c r="E53" s="24" t="n"/>
+      <c r="F53" s="24" t="n"/>
+      <c r="G53" s="24" t="n"/>
+      <c r="H53" s="24" t="n"/>
+      <c r="I53" s="24" t="n"/>
+      <c r="J53" s="24" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="23" t="n"/>
-      <c r="C54" s="23" t="n"/>
-      <c r="D54" s="23" t="n"/>
-      <c r="E54" s="23" t="n"/>
-      <c r="F54" s="23" t="n"/>
-      <c r="G54" s="23" t="n"/>
-      <c r="H54" s="23" t="n"/>
-      <c r="I54" s="23" t="n"/>
-      <c r="J54" s="23" t="n"/>
+      <c r="B54" s="24" t="n"/>
+      <c r="C54" s="24" t="n"/>
+      <c r="D54" s="24" t="n"/>
+      <c r="E54" s="24" t="n"/>
+      <c r="F54" s="24" t="n"/>
+      <c r="G54" s="24" t="n"/>
+      <c r="H54" s="24" t="n"/>
+      <c r="I54" s="24" t="n"/>
+      <c r="J54" s="24" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="23" t="n"/>
-      <c r="C55" s="23" t="n"/>
-      <c r="D55" s="23" t="n"/>
-      <c r="E55" s="23" t="n"/>
-      <c r="F55" s="23" t="n"/>
-      <c r="G55" s="23" t="n"/>
-      <c r="H55" s="23" t="n"/>
-      <c r="I55" s="23" t="n"/>
-      <c r="J55" s="23" t="n"/>
+      <c r="B55" s="24" t="n"/>
+      <c r="C55" s="24" t="n"/>
+      <c r="D55" s="24" t="n"/>
+      <c r="E55" s="24" t="n"/>
+      <c r="F55" s="24" t="n"/>
+      <c r="G55" s="24" t="n"/>
+      <c r="H55" s="24" t="n"/>
+      <c r="I55" s="24" t="n"/>
+      <c r="J55" s="24" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="23" t="n"/>
-      <c r="C56" s="23" t="n"/>
-      <c r="D56" s="23" t="n"/>
-      <c r="E56" s="23" t="n"/>
-      <c r="F56" s="23" t="n"/>
-      <c r="G56" s="23" t="n"/>
-      <c r="H56" s="23" t="n"/>
-      <c r="I56" s="23" t="n"/>
-      <c r="J56" s="23" t="n"/>
+      <c r="B56" s="24" t="n"/>
+      <c r="C56" s="24" t="n"/>
+      <c r="D56" s="24" t="n"/>
+      <c r="E56" s="24" t="n"/>
+      <c r="F56" s="24" t="n"/>
+      <c r="G56" s="24" t="n"/>
+      <c r="H56" s="24" t="n"/>
+      <c r="I56" s="24" t="n"/>
+      <c r="J56" s="24" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="23" t="n"/>
-      <c r="C57" s="23" t="n"/>
-      <c r="D57" s="23" t="n"/>
-      <c r="E57" s="23" t="n"/>
-      <c r="F57" s="23" t="n"/>
-      <c r="G57" s="23" t="n"/>
-      <c r="H57" s="23" t="n"/>
-      <c r="I57" s="23" t="n"/>
-      <c r="J57" s="23" t="n"/>
+      <c r="B57" s="24" t="n"/>
+      <c r="C57" s="24" t="n"/>
+      <c r="D57" s="24" t="n"/>
+      <c r="E57" s="24" t="n"/>
+      <c r="F57" s="24" t="n"/>
+      <c r="G57" s="24" t="n"/>
+      <c r="H57" s="24" t="n"/>
+      <c r="I57" s="24" t="n"/>
+      <c r="J57" s="24" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="23" t="n"/>
-      <c r="C58" s="23" t="n"/>
-      <c r="D58" s="23" t="n"/>
-      <c r="E58" s="23" t="n"/>
-      <c r="F58" s="23" t="n"/>
-      <c r="G58" s="23" t="n"/>
-      <c r="H58" s="23" t="n"/>
-      <c r="I58" s="23" t="n"/>
-      <c r="J58" s="23" t="n"/>
+      <c r="B58" s="24" t="n"/>
+      <c r="C58" s="24" t="n"/>
+      <c r="D58" s="24" t="n"/>
+      <c r="E58" s="24" t="n"/>
+      <c r="F58" s="24" t="n"/>
+      <c r="G58" s="24" t="n"/>
+      <c r="H58" s="24" t="n"/>
+      <c r="I58" s="24" t="n"/>
+      <c r="J58" s="24" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="23" t="n"/>
-      <c r="C59" s="23" t="n"/>
-      <c r="D59" s="23" t="n"/>
-      <c r="E59" s="23" t="n"/>
-      <c r="F59" s="23" t="n"/>
-      <c r="G59" s="23" t="n"/>
-      <c r="H59" s="23" t="n"/>
-      <c r="I59" s="23" t="n"/>
-      <c r="J59" s="23" t="n"/>
+      <c r="B59" s="24" t="n"/>
+      <c r="C59" s="24" t="n"/>
+      <c r="D59" s="24" t="n"/>
+      <c r="E59" s="24" t="n"/>
+      <c r="F59" s="24" t="n"/>
+      <c r="G59" s="24" t="n"/>
+      <c r="H59" s="24" t="n"/>
+      <c r="I59" s="24" t="n"/>
+      <c r="J59" s="24" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="23" t="n"/>
-      <c r="C60" s="23" t="n"/>
-      <c r="D60" s="23" t="n"/>
-      <c r="E60" s="23" t="n"/>
-      <c r="F60" s="23" t="n"/>
-      <c r="G60" s="23" t="n"/>
-      <c r="H60" s="23" t="n"/>
-      <c r="I60" s="23" t="n"/>
-      <c r="J60" s="23" t="n"/>
+      <c r="B60" s="24" t="n"/>
+      <c r="C60" s="24" t="n"/>
+      <c r="D60" s="24" t="n"/>
+      <c r="E60" s="24" t="n"/>
+      <c r="F60" s="24" t="n"/>
+      <c r="G60" s="24" t="n"/>
+      <c r="H60" s="24" t="n"/>
+      <c r="I60" s="24" t="n"/>
+      <c r="J60" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2776,7 +3874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2789,6 +3887,11 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -2919,7 +4022,7 @@
       <c r="F20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="25" t="n">
+      <c r="G20" s="26" t="n">
         <v>-1</v>
       </c>
       <c r="H20" s="10" t="n">
@@ -2952,7 +4055,7 @@
       <c r="F21" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="25" t="n">
+      <c r="G21" s="26" t="n">
         <v>3</v>
       </c>
       <c r="H21" s="10" t="n">
@@ -2985,7 +4088,7 @@
       <c r="F22" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="25" t="n">
+      <c r="G22" s="26" t="n">
         <v>-6</v>
       </c>
       <c r="H22" s="10" t="n">
@@ -3041,7 +4144,7 @@
       <c r="F24" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="G24" s="26" t="n">
+      <c r="G24" s="27" t="n">
         <v>-5</v>
       </c>
       <c r="H24" s="16" t="n">
@@ -3052,17 +4155,54 @@
       </c>
       <c r="J24" s="16" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="26"/>
+    <row r="25">
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>TABLA DE PUNTOS PARA EL GRÁFICO NATIVO DE EXCEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="L26" s="19" t="inlineStr">
+        <is>
+          <t>x_val</t>
+        </is>
+      </c>
+      <c r="M26" s="19" t="inlineStr">
+        <is>
+          <t>R1 (x2&gt;=2)</t>
+        </is>
+      </c>
+      <c r="N26" s="19" t="inlineStr">
+        <is>
+          <t>R2 (4x1+6x2&gt;=24)</t>
+        </is>
+      </c>
+      <c r="O26" s="19" t="inlineStr">
+        <is>
+          <t>R3 (10x1-30x2&gt;=30)</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
           <t>3. RESPUESTAS A LAS PREGUNTAS TEÓRICAS Y CONCLUSIÓN DEL CASO</t>
         </is>
       </c>
+      <c r="L27" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N27" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="O27" s="10" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>• Respuesta a) Formulación Deducida:
    Variables: X1 = Toneladas diarias de PET reciclado | X2 = Toneladas diarias de Polietileno procesado.
@@ -3080,157 +4220,205 @@
    3. Techo presupuestario del municipio para el pago de subsidios o saturación de la demanda comercial.</t>
         </is>
       </c>
-      <c r="C28" s="23" t="n"/>
-      <c r="D28" s="23" t="n"/>
-      <c r="E28" s="23" t="n"/>
-      <c r="F28" s="23" t="n"/>
-      <c r="G28" s="23" t="n"/>
-      <c r="H28" s="23" t="n"/>
-      <c r="I28" s="23" t="n"/>
-      <c r="J28" s="23" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
+      <c r="F28" s="24" t="n"/>
+      <c r="G28" s="24" t="n"/>
+      <c r="H28" s="24" t="n"/>
+      <c r="I28" s="24" t="n"/>
+      <c r="J28" s="24" t="n"/>
+      <c r="L28" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="M28" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N28" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="O28" s="20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
-      <c r="B29" s="23" t="n"/>
-      <c r="C29" s="23" t="n"/>
-      <c r="D29" s="23" t="n"/>
-      <c r="E29" s="23" t="n"/>
-      <c r="F29" s="23" t="n"/>
-      <c r="G29" s="23" t="n"/>
-      <c r="H29" s="23" t="n"/>
-      <c r="I29" s="23" t="n"/>
-      <c r="J29" s="23" t="n"/>
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
+      <c r="F29" s="24" t="n"/>
+      <c r="G29" s="24" t="n"/>
+      <c r="H29" s="24" t="n"/>
+      <c r="I29" s="24" t="n"/>
+      <c r="J29" s="24" t="n"/>
+      <c r="L29" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="M29" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N29" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
-      <c r="B30" s="23" t="n"/>
-      <c r="C30" s="23" t="n"/>
-      <c r="D30" s="23" t="n"/>
-      <c r="E30" s="23" t="n"/>
-      <c r="F30" s="23" t="n"/>
-      <c r="G30" s="23" t="n"/>
-      <c r="H30" s="23" t="n"/>
-      <c r="I30" s="23" t="n"/>
-      <c r="J30" s="23" t="n"/>
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="24" t="n"/>
+      <c r="F30" s="24" t="n"/>
+      <c r="G30" s="24" t="n"/>
+      <c r="H30" s="24" t="n"/>
+      <c r="I30" s="24" t="n"/>
+      <c r="J30" s="24" t="n"/>
+      <c r="L30" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="M30" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N30" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="20" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="31">
-      <c r="B31" s="23" t="n"/>
-      <c r="C31" s="23" t="n"/>
-      <c r="D31" s="23" t="n"/>
-      <c r="E31" s="23" t="n"/>
-      <c r="F31" s="23" t="n"/>
-      <c r="G31" s="23" t="n"/>
-      <c r="H31" s="23" t="n"/>
-      <c r="I31" s="23" t="n"/>
-      <c r="J31" s="23" t="n"/>
+      <c r="B31" s="24" t="n"/>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="24" t="n"/>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="24" t="n"/>
+      <c r="J31" s="24" t="n"/>
+      <c r="L31" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="M31" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="20" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="32">
-      <c r="B32" s="23" t="n"/>
-      <c r="C32" s="23" t="n"/>
-      <c r="D32" s="23" t="n"/>
-      <c r="E32" s="23" t="n"/>
-      <c r="F32" s="23" t="n"/>
-      <c r="G32" s="23" t="n"/>
-      <c r="H32" s="23" t="n"/>
-      <c r="I32" s="23" t="n"/>
-      <c r="J32" s="23" t="n"/>
+      <c r="B32" s="24" t="n"/>
+      <c r="C32" s="24" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="24" t="n"/>
+      <c r="H32" s="24" t="n"/>
+      <c r="I32" s="24" t="n"/>
+      <c r="J32" s="24" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="23" t="n"/>
-      <c r="C33" s="23" t="n"/>
-      <c r="D33" s="23" t="n"/>
-      <c r="E33" s="23" t="n"/>
-      <c r="F33" s="23" t="n"/>
-      <c r="G33" s="23" t="n"/>
-      <c r="H33" s="23" t="n"/>
-      <c r="I33" s="23" t="n"/>
-      <c r="J33" s="23" t="n"/>
+      <c r="B33" s="24" t="n"/>
+      <c r="C33" s="24" t="n"/>
+      <c r="D33" s="24" t="n"/>
+      <c r="E33" s="24" t="n"/>
+      <c r="F33" s="24" t="n"/>
+      <c r="G33" s="24" t="n"/>
+      <c r="H33" s="24" t="n"/>
+      <c r="I33" s="24" t="n"/>
+      <c r="J33" s="24" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="23" t="n"/>
-      <c r="C34" s="23" t="n"/>
-      <c r="D34" s="23" t="n"/>
-      <c r="E34" s="23" t="n"/>
-      <c r="F34" s="23" t="n"/>
-      <c r="G34" s="23" t="n"/>
-      <c r="H34" s="23" t="n"/>
-      <c r="I34" s="23" t="n"/>
-      <c r="J34" s="23" t="n"/>
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="24" t="n"/>
+      <c r="F34" s="24" t="n"/>
+      <c r="G34" s="24" t="n"/>
+      <c r="H34" s="24" t="n"/>
+      <c r="I34" s="24" t="n"/>
+      <c r="J34" s="24" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="23" t="n"/>
-      <c r="C35" s="23" t="n"/>
-      <c r="D35" s="23" t="n"/>
-      <c r="E35" s="23" t="n"/>
-      <c r="F35" s="23" t="n"/>
-      <c r="G35" s="23" t="n"/>
-      <c r="H35" s="23" t="n"/>
-      <c r="I35" s="23" t="n"/>
-      <c r="J35" s="23" t="n"/>
+      <c r="B35" s="24" t="n"/>
+      <c r="C35" s="24" t="n"/>
+      <c r="D35" s="24" t="n"/>
+      <c r="E35" s="24" t="n"/>
+      <c r="F35" s="24" t="n"/>
+      <c r="G35" s="24" t="n"/>
+      <c r="H35" s="24" t="n"/>
+      <c r="I35" s="24" t="n"/>
+      <c r="J35" s="24" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="23" t="n"/>
-      <c r="C36" s="23" t="n"/>
-      <c r="D36" s="23" t="n"/>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="23" t="n"/>
-      <c r="G36" s="23" t="n"/>
-      <c r="H36" s="23" t="n"/>
-      <c r="I36" s="23" t="n"/>
-      <c r="J36" s="23" t="n"/>
+      <c r="B36" s="24" t="n"/>
+      <c r="C36" s="24" t="n"/>
+      <c r="D36" s="24" t="n"/>
+      <c r="E36" s="24" t="n"/>
+      <c r="F36" s="24" t="n"/>
+      <c r="G36" s="24" t="n"/>
+      <c r="H36" s="24" t="n"/>
+      <c r="I36" s="24" t="n"/>
+      <c r="J36" s="24" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="23" t="n"/>
-      <c r="C37" s="23" t="n"/>
-      <c r="D37" s="23" t="n"/>
-      <c r="E37" s="23" t="n"/>
-      <c r="F37" s="23" t="n"/>
-      <c r="G37" s="23" t="n"/>
-      <c r="H37" s="23" t="n"/>
-      <c r="I37" s="23" t="n"/>
-      <c r="J37" s="23" t="n"/>
+      <c r="B37" s="24" t="n"/>
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="n"/>
+      <c r="E37" s="24" t="n"/>
+      <c r="F37" s="24" t="n"/>
+      <c r="G37" s="24" t="n"/>
+      <c r="H37" s="24" t="n"/>
+      <c r="I37" s="24" t="n"/>
+      <c r="J37" s="24" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="23" t="n"/>
-      <c r="C38" s="23" t="n"/>
-      <c r="D38" s="23" t="n"/>
-      <c r="E38" s="23" t="n"/>
-      <c r="F38" s="23" t="n"/>
-      <c r="G38" s="23" t="n"/>
-      <c r="H38" s="23" t="n"/>
-      <c r="I38" s="23" t="n"/>
-      <c r="J38" s="23" t="n"/>
+      <c r="B38" s="24" t="n"/>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="24" t="n"/>
+      <c r="G38" s="24" t="n"/>
+      <c r="H38" s="24" t="n"/>
+      <c r="I38" s="24" t="n"/>
+      <c r="J38" s="24" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="23" t="n"/>
-      <c r="C39" s="23" t="n"/>
-      <c r="D39" s="23" t="n"/>
-      <c r="E39" s="23" t="n"/>
-      <c r="F39" s="23" t="n"/>
-      <c r="G39" s="23" t="n"/>
-      <c r="H39" s="23" t="n"/>
-      <c r="I39" s="23" t="n"/>
-      <c r="J39" s="23" t="n"/>
+      <c r="B39" s="24" t="n"/>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="24" t="n"/>
+      <c r="H39" s="24" t="n"/>
+      <c r="I39" s="24" t="n"/>
+      <c r="J39" s="24" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="23" t="n"/>
-      <c r="C40" s="23" t="n"/>
-      <c r="D40" s="23" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
-      <c r="I40" s="23" t="n"/>
-      <c r="J40" s="23" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="24" t="n"/>
+      <c r="H40" s="24" t="n"/>
+      <c r="I40" s="24" t="n"/>
+      <c r="J40" s="24" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="23" t="n"/>
-      <c r="C41" s="23" t="n"/>
-      <c r="D41" s="23" t="n"/>
-      <c r="E41" s="23" t="n"/>
-      <c r="F41" s="23" t="n"/>
-      <c r="G41" s="23" t="n"/>
-      <c r="H41" s="23" t="n"/>
-      <c r="I41" s="23" t="n"/>
-      <c r="J41" s="23" t="n"/>
+      <c r="B41" s="24" t="n"/>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="24" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="24" t="n"/>
+      <c r="G41" s="24" t="n"/>
+      <c r="H41" s="24" t="n"/>
+      <c r="I41" s="24" t="n"/>
+      <c r="J41" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3249,7 +4437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3262,6 +4450,11 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -3370,7 +4563,7 @@
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>μ3</t>
+          <t>Θ</t>
         </is>
       </c>
     </row>
@@ -3440,12 +4633,12 @@
       <c r="B22" s="8" t="n">
         <v>-1000</v>
       </c>
-      <c r="C22" s="27" t="inlineStr">
+      <c r="C22" s="28" t="inlineStr">
         <is>
           <t>μ3</t>
         </is>
       </c>
-      <c r="D22" s="24" t="n">
+      <c r="D22" s="25" t="n">
         <v>7.33</v>
       </c>
       <c r="E22" s="10" t="n">
@@ -3478,7 +4671,7 @@
           <t>=</t>
         </is>
       </c>
-      <c r="D23" s="28" t="inlineStr">
+      <c r="D23" s="29" t="inlineStr">
         <is>
           <t>0.33 - 7.33M</t>
         </is>
@@ -3502,48 +4695,87 @@
         </is>
       </c>
       <c r="D24" s="16" t="n"/>
-      <c r="E24" s="29" t="inlineStr">
+      <c r="E24" s="30" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="F24" s="29" t="inlineStr">
+      <c r="F24" s="30" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="G24" s="29" t="inlineStr">
+      <c r="G24" s="30" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="H24" s="29" t="inlineStr">
+      <c r="H24" s="30" t="inlineStr">
         <is>
           <t>0.33 + 0.67M</t>
         </is>
       </c>
-      <c r="I24" s="29" t="inlineStr">
+      <c r="I24" s="30" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="J24" s="29" t="inlineStr">
+      <c r="J24" s="30" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
+    <row r="25">
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>TABLA DE PUNTOS PARA EL GRÁFICO NATIVO DE EXCEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="L26" s="19" t="inlineStr">
+        <is>
+          <t>x_val</t>
+        </is>
+      </c>
+      <c r="M26" s="19" t="inlineStr">
+        <is>
+          <t>R1 (x1+x2&lt;=6)</t>
+        </is>
+      </c>
+      <c r="N26" s="19" t="inlineStr">
+        <is>
+          <t>R2 (2x1+3x2&lt;=1)</t>
+        </is>
+      </c>
+      <c r="O26" s="19" t="inlineStr">
+        <is>
+          <t>R3 (-x1+2x2&gt;=8)</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
       <c r="B27" s="3" t="inlineStr">
         <is>
           <t>3. RESPUESTAS A LAS PREGUNTAS TEÓRICAS Y CONCLUSIÓN DEL CASO</t>
         </is>
       </c>
+      <c r="L27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N27" s="9" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="O27" s="9" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>• Respuesta a) Formulación Deducida:
    Variables: X1 = Camisas confeccionadas | X2 = Pantalones confeccionados.
@@ -3561,157 +4793,189 @@
    4. Diagnóstico de Examen: PROBLEMA INCOMPATIBLE (Infactible). La gerencia debe renegociar el contrato o ampliar el presupuesto de caja.</t>
         </is>
       </c>
-      <c r="C28" s="23" t="n"/>
-      <c r="D28" s="23" t="n"/>
-      <c r="E28" s="23" t="n"/>
-      <c r="F28" s="23" t="n"/>
-      <c r="G28" s="23" t="n"/>
-      <c r="H28" s="23" t="n"/>
-      <c r="I28" s="23" t="n"/>
-      <c r="J28" s="23" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
+      <c r="F28" s="24" t="n"/>
+      <c r="G28" s="24" t="n"/>
+      <c r="H28" s="24" t="n"/>
+      <c r="I28" s="24" t="n"/>
+      <c r="J28" s="24" t="n"/>
+      <c r="L28" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M28" s="9" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="N28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="9" t="n">
+        <v>4.25</v>
+      </c>
     </row>
     <row r="29">
-      <c r="B29" s="23" t="n"/>
-      <c r="C29" s="23" t="n"/>
-      <c r="D29" s="23" t="n"/>
-      <c r="E29" s="23" t="n"/>
-      <c r="F29" s="23" t="n"/>
-      <c r="G29" s="23" t="n"/>
-      <c r="H29" s="23" t="n"/>
-      <c r="I29" s="23" t="n"/>
-      <c r="J29" s="23" t="n"/>
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
+      <c r="F29" s="24" t="n"/>
+      <c r="G29" s="24" t="n"/>
+      <c r="H29" s="24" t="n"/>
+      <c r="I29" s="24" t="n"/>
+      <c r="J29" s="24" t="n"/>
+      <c r="L29" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N29" s="10" t="n"/>
+      <c r="O29" s="9" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="30">
-      <c r="B30" s="23" t="n"/>
-      <c r="C30" s="23" t="n"/>
-      <c r="D30" s="23" t="n"/>
-      <c r="E30" s="23" t="n"/>
-      <c r="F30" s="23" t="n"/>
-      <c r="G30" s="23" t="n"/>
-      <c r="H30" s="23" t="n"/>
-      <c r="I30" s="23" t="n"/>
-      <c r="J30" s="23" t="n"/>
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="24" t="n"/>
+      <c r="F30" s="24" t="n"/>
+      <c r="G30" s="24" t="n"/>
+      <c r="H30" s="24" t="n"/>
+      <c r="I30" s="24" t="n"/>
+      <c r="J30" s="24" t="n"/>
+      <c r="L30" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="10" t="n"/>
+      <c r="O30" s="9" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="31">
-      <c r="B31" s="23" t="n"/>
-      <c r="C31" s="23" t="n"/>
-      <c r="D31" s="23" t="n"/>
-      <c r="E31" s="23" t="n"/>
-      <c r="F31" s="23" t="n"/>
-      <c r="G31" s="23" t="n"/>
-      <c r="H31" s="23" t="n"/>
-      <c r="I31" s="23" t="n"/>
-      <c r="J31" s="23" t="n"/>
+      <c r="B31" s="24" t="n"/>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="24" t="n"/>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="24" t="n"/>
+      <c r="J31" s="24" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="23" t="n"/>
-      <c r="C32" s="23" t="n"/>
-      <c r="D32" s="23" t="n"/>
-      <c r="E32" s="23" t="n"/>
-      <c r="F32" s="23" t="n"/>
-      <c r="G32" s="23" t="n"/>
-      <c r="H32" s="23" t="n"/>
-      <c r="I32" s="23" t="n"/>
-      <c r="J32" s="23" t="n"/>
+      <c r="B32" s="24" t="n"/>
+      <c r="C32" s="24" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="24" t="n"/>
+      <c r="H32" s="24" t="n"/>
+      <c r="I32" s="24" t="n"/>
+      <c r="J32" s="24" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="23" t="n"/>
-      <c r="C33" s="23" t="n"/>
-      <c r="D33" s="23" t="n"/>
-      <c r="E33" s="23" t="n"/>
-      <c r="F33" s="23" t="n"/>
-      <c r="G33" s="23" t="n"/>
-      <c r="H33" s="23" t="n"/>
-      <c r="I33" s="23" t="n"/>
-      <c r="J33" s="23" t="n"/>
+      <c r="B33" s="24" t="n"/>
+      <c r="C33" s="24" t="n"/>
+      <c r="D33" s="24" t="n"/>
+      <c r="E33" s="24" t="n"/>
+      <c r="F33" s="24" t="n"/>
+      <c r="G33" s="24" t="n"/>
+      <c r="H33" s="24" t="n"/>
+      <c r="I33" s="24" t="n"/>
+      <c r="J33" s="24" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="23" t="n"/>
-      <c r="C34" s="23" t="n"/>
-      <c r="D34" s="23" t="n"/>
-      <c r="E34" s="23" t="n"/>
-      <c r="F34" s="23" t="n"/>
-      <c r="G34" s="23" t="n"/>
-      <c r="H34" s="23" t="n"/>
-      <c r="I34" s="23" t="n"/>
-      <c r="J34" s="23" t="n"/>
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="24" t="n"/>
+      <c r="F34" s="24" t="n"/>
+      <c r="G34" s="24" t="n"/>
+      <c r="H34" s="24" t="n"/>
+      <c r="I34" s="24" t="n"/>
+      <c r="J34" s="24" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="23" t="n"/>
-      <c r="C35" s="23" t="n"/>
-      <c r="D35" s="23" t="n"/>
-      <c r="E35" s="23" t="n"/>
-      <c r="F35" s="23" t="n"/>
-      <c r="G35" s="23" t="n"/>
-      <c r="H35" s="23" t="n"/>
-      <c r="I35" s="23" t="n"/>
-      <c r="J35" s="23" t="n"/>
+      <c r="B35" s="24" t="n"/>
+      <c r="C35" s="24" t="n"/>
+      <c r="D35" s="24" t="n"/>
+      <c r="E35" s="24" t="n"/>
+      <c r="F35" s="24" t="n"/>
+      <c r="G35" s="24" t="n"/>
+      <c r="H35" s="24" t="n"/>
+      <c r="I35" s="24" t="n"/>
+      <c r="J35" s="24" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="23" t="n"/>
-      <c r="C36" s="23" t="n"/>
-      <c r="D36" s="23" t="n"/>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="23" t="n"/>
-      <c r="G36" s="23" t="n"/>
-      <c r="H36" s="23" t="n"/>
-      <c r="I36" s="23" t="n"/>
-      <c r="J36" s="23" t="n"/>
+      <c r="B36" s="24" t="n"/>
+      <c r="C36" s="24" t="n"/>
+      <c r="D36" s="24" t="n"/>
+      <c r="E36" s="24" t="n"/>
+      <c r="F36" s="24" t="n"/>
+      <c r="G36" s="24" t="n"/>
+      <c r="H36" s="24" t="n"/>
+      <c r="I36" s="24" t="n"/>
+      <c r="J36" s="24" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="23" t="n"/>
-      <c r="C37" s="23" t="n"/>
-      <c r="D37" s="23" t="n"/>
-      <c r="E37" s="23" t="n"/>
-      <c r="F37" s="23" t="n"/>
-      <c r="G37" s="23" t="n"/>
-      <c r="H37" s="23" t="n"/>
-      <c r="I37" s="23" t="n"/>
-      <c r="J37" s="23" t="n"/>
+      <c r="B37" s="24" t="n"/>
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="n"/>
+      <c r="E37" s="24" t="n"/>
+      <c r="F37" s="24" t="n"/>
+      <c r="G37" s="24" t="n"/>
+      <c r="H37" s="24" t="n"/>
+      <c r="I37" s="24" t="n"/>
+      <c r="J37" s="24" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="23" t="n"/>
-      <c r="C38" s="23" t="n"/>
-      <c r="D38" s="23" t="n"/>
-      <c r="E38" s="23" t="n"/>
-      <c r="F38" s="23" t="n"/>
-      <c r="G38" s="23" t="n"/>
-      <c r="H38" s="23" t="n"/>
-      <c r="I38" s="23" t="n"/>
-      <c r="J38" s="23" t="n"/>
+      <c r="B38" s="24" t="n"/>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="24" t="n"/>
+      <c r="G38" s="24" t="n"/>
+      <c r="H38" s="24" t="n"/>
+      <c r="I38" s="24" t="n"/>
+      <c r="J38" s="24" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="23" t="n"/>
-      <c r="C39" s="23" t="n"/>
-      <c r="D39" s="23" t="n"/>
-      <c r="E39" s="23" t="n"/>
-      <c r="F39" s="23" t="n"/>
-      <c r="G39" s="23" t="n"/>
-      <c r="H39" s="23" t="n"/>
-      <c r="I39" s="23" t="n"/>
-      <c r="J39" s="23" t="n"/>
+      <c r="B39" s="24" t="n"/>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="24" t="n"/>
+      <c r="H39" s="24" t="n"/>
+      <c r="I39" s="24" t="n"/>
+      <c r="J39" s="24" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="23" t="n"/>
-      <c r="C40" s="23" t="n"/>
-      <c r="D40" s="23" t="n"/>
-      <c r="E40" s="23" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="23" t="n"/>
-      <c r="I40" s="23" t="n"/>
-      <c r="J40" s="23" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="24" t="n"/>
+      <c r="H40" s="24" t="n"/>
+      <c r="I40" s="24" t="n"/>
+      <c r="J40" s="24" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="23" t="n"/>
-      <c r="C41" s="23" t="n"/>
-      <c r="D41" s="23" t="n"/>
-      <c r="E41" s="23" t="n"/>
-      <c r="F41" s="23" t="n"/>
-      <c r="G41" s="23" t="n"/>
-      <c r="H41" s="23" t="n"/>
-      <c r="I41" s="23" t="n"/>
-      <c r="J41" s="23" t="n"/>
+      <c r="B41" s="24" t="n"/>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="24" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="24" t="n"/>
+      <c r="G41" s="24" t="n"/>
+      <c r="H41" s="24" t="n"/>
+      <c r="I41" s="24" t="n"/>
+      <c r="J41" s="24" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>